<commit_message>
Docs sweep for PIN login + client docs finalised without proposed items
- Client docs: CLIENT_FEATURES.md + Feature-Summary.docx updated for the PIN
  sign-in and the operative Shop Floor app (new sections, 14 modules);
  Feature-Tracker.xlsx: Factory PIN sign-in row, manager-set PINs, new Shop
  Floor module (4 rows) - now 73 Completed / 0 Planned / 0 Proposed
- Per client-facing preference: removed all Proposed/upsell content from the
  doc, docx and tracker (ideas remain in DEVLOG for future quoting)
- Consistency sweep: README auth section, DEPLOY.md (no more Supabase user
  creation), .env.example comments, PROJECT_PLAN.md annotations; deleted
  obsolete create-user script + npm entry

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/docs/Bowson-GRP-Feature-Tracker.xlsx
+++ b/docs/Bowson-GRP-Feature-Tracker.xlsx
@@ -20,7 +20,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="313" uniqueCount="179">
   <si>
     <t>#</t>
   </si>
@@ -52,18 +52,9 @@
     <t>Completed</t>
   </si>
   <si>
-    <t>Secure login accounts</t>
-  </si>
-  <si>
-    <t>Every user signs in with their own account.</t>
-  </si>
-  <si>
     <t>Role-based access levels</t>
   </si>
   <si>
-    <t>Admin, Manager and Operative levels. Operatives can work tickets on the shop floor but cannot create or delete orders, change settings or edit the catalogue.</t>
-  </si>
-  <si>
     <t>Manager PIN protection</t>
   </si>
   <si>
@@ -526,62 +517,53 @@
     <t>4. Once a proposed feature is agreed and delivered, its status changes to Completed.</t>
   </si>
   <si>
-    <t>Included</t>
-  </si>
-  <si>
-    <t>Delivered 11/07/2026 - maintenance moulds now hidden in the order-page and ticket-popup mould dropdowns (the currently-assigned mould stays visible).</t>
-  </si>
-  <si>
-    <t>Delivered 11/07/2026 - register Status column now shows live Free/Partial/Full/Maintenance with an In use count, matching the mould board.</t>
-  </si>
-  <si>
-    <t>Recommended enhancements</t>
-  </si>
-  <si>
-    <t>Server-side enforcement of Packing &amp; QC gates</t>
-  </si>
-  <si>
-    <t>The packing-checklist and QC-reference rules are enforced in the app screens today (as in the original tool). Add matching enforcement in the backend so the rules also hold for bulk actions and any future integrations.</t>
-  </si>
-  <si>
-    <t>Proposed</t>
-  </si>
-  <si>
-    <t>Quote on request</t>
-  </si>
-  <si>
-    <t>Optional - app already matches the original tool; this is a further improvement.</t>
-  </si>
-  <si>
-    <t>Report skipped tickets in bulk advance</t>
-  </si>
-  <si>
-    <t>When a bulk stage-move skips tickets that are blocked by a rule, list exactly which ones were skipped and why (currently it reports only the moved count).</t>
-  </si>
-  <si>
-    <t>PIN-protect single ticket deletion</t>
-  </si>
-  <si>
-    <t>Deleting a whole order already needs the manager PIN; extend the same protection to deleting an individual ticket.</t>
-  </si>
-  <si>
-    <t>Live cure countdown on the Mould board</t>
-  </si>
-  <si>
-    <t>Cure timers tick live on the T-Card board; make them tick live on the Mould board view too.</t>
-  </si>
-  <si>
-    <t>Include customers in global search</t>
-  </si>
-  <si>
-    <t>The top-bar search covers orders and tickets; add customers so a customer name jumps straight to their record.</t>
+    <t>Factory PIN sign-in</t>
+  </si>
+  <si>
+    <t>Tap-your-name sign-in screen: every operative appears as a card (with a live On Shift indicator) plus a Manager Login button, then a big-button PIN pad. Designed for a shared workshop screen or tablet - no usernames or email addresses.</t>
+  </si>
+  <si>
+    <t>Manager-set operative PINs</t>
+  </si>
+  <si>
+    <t>Each operative has their own sign-in PIN, set by the manager in the operative profile (default 1234 until set). The manager PIN itself is changeable in Settings. PINs are never visible to operatives.</t>
+  </si>
+  <si>
+    <t>Shop Floor (Operative App)</t>
+  </si>
+  <si>
+    <t>My Tickets with live time tracking</t>
+  </si>
+  <si>
+    <t>Operatives see the jobs they are clocked onto, each with a live running timer, Pause, and one-tap Stage Done that moves the job on and stops the clock. Cure countdowns show a Ready-Advance prompt; a Completed Today list totals hours logged.</t>
+  </si>
+  <si>
+    <t>Available work - tap to join</t>
+  </si>
+  <si>
+    <t>The queue of tickets at the operative's allocated stages (from their skills profile). One tap on Join assigns them and starts their timer; shows who else is already working on each job.</t>
+  </si>
+  <si>
+    <t>Shop-floor board (read-only)</t>
+  </si>
+  <si>
+    <t>A live stage-by-stage view of the whole board showing who is working on what right now.</t>
+  </si>
+  <si>
+    <t>End Shift and sign-out safeguards</t>
+  </si>
+  <si>
+    <t>One tap stops all the operative's running timers; signing out with timers still running asks first so no time is lost.</t>
+  </si>
+  <si>
+    <t xml:space="preserve"> Manager and Operative levels. Operatives can work tickets on the shop floor but cannot create or delete orders, change settings or edit the catalogue.</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <fonts count="7">
+  <fonts count="6">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -628,16 +610,8 @@
       <family val="2"/>
       <scheme val="minor"/>
     </font>
-    <font>
-      <b/>
-      <sz val="11"/>
-      <color rgb="FF1559A0"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
   </fonts>
-  <fills count="5">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -653,12 +627,6 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFDFF2EB"/>
-        <bgColor indexed="64"/>
-      </patternFill>
-    </fill>
-    <fill>
-      <patternFill patternType="solid">
-        <fgColor rgb="FFE8F1FA"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -690,7 +658,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="15">
+  <cellXfs count="12">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
@@ -715,15 +683,6 @@
     <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="4" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="top"/>
-    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -1018,15 +977,15 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:G74"/>
+  <dimension ref="A1:F74"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
-    <col min="1" max="1" width="5.7109375" customWidth="1"/>
-    <col min="2" max="2" width="20.7109375" customWidth="1"/>
-    <col min="3" max="3" width="34.7109375" customWidth="1"/>
+    <col min="1" max="1" width="4.28515625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="25.7109375" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="40.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="72.7109375" style="3" customWidth="1"/>
-    <col min="5" max="5" width="12.7109375" customWidth="1"/>
-    <col min="6" max="6" width="34.7109375" style="3" customWidth="1"/>
+    <col min="5" max="5" width="19.140625" customWidth="1"/>
+    <col min="6" max="6" width="15.5703125" style="3" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:6">
@@ -1067,7 +1026,7 @@
       </c>
       <c r="F2" s="7"/>
     </row>
-    <row r="3" spans="1:6">
+    <row r="3" spans="1:6" ht="60">
       <c r="A3" s="6">
         <v>2</v>
       </c>
@@ -1075,10 +1034,10 @@
         <v>6</v>
       </c>
       <c r="C3" s="6" t="s">
-        <v>10</v>
+        <v>165</v>
       </c>
       <c r="D3" s="7" t="s">
-        <v>11</v>
+        <v>166</v>
       </c>
       <c r="E3" s="8" t="s">
         <v>9</v>
@@ -1093,10 +1052,10 @@
         <v>6</v>
       </c>
       <c r="C4" s="6" t="s">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="D4" s="7" t="s">
-        <v>13</v>
+        <v>178</v>
       </c>
       <c r="E4" s="8" t="s">
         <v>9</v>
@@ -1111,10 +1070,10 @@
         <v>6</v>
       </c>
       <c r="C5" s="6" t="s">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="D5" s="7" t="s">
-        <v>15</v>
+        <v>12</v>
       </c>
       <c r="E5" s="8" t="s">
         <v>9</v>
@@ -1129,28 +1088,28 @@
         <v>6</v>
       </c>
       <c r="C6" s="6" t="s">
-        <v>16</v>
+        <v>13</v>
       </c>
       <c r="D6" s="7" t="s">
-        <v>17</v>
+        <v>14</v>
       </c>
       <c r="E6" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F6" s="7"/>
     </row>
-    <row r="7" spans="1:6" ht="30">
+    <row r="7" spans="1:6" ht="45">
       <c r="A7" s="6">
         <v>6</v>
       </c>
       <c r="B7" s="6" t="s">
-        <v>18</v>
+        <v>6</v>
       </c>
       <c r="C7" s="6" t="s">
-        <v>19</v>
+        <v>167</v>
       </c>
       <c r="D7" s="7" t="s">
-        <v>20</v>
+        <v>168</v>
       </c>
       <c r="E7" s="8" t="s">
         <v>9</v>
@@ -1162,31 +1121,31 @@
         <v>7</v>
       </c>
       <c r="B8" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C8" s="6" t="s">
-        <v>21</v>
+        <v>16</v>
       </c>
       <c r="D8" s="7" t="s">
-        <v>22</v>
+        <v>17</v>
       </c>
       <c r="E8" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F8" s="7"/>
     </row>
-    <row r="9" spans="1:6">
+    <row r="9" spans="1:6" ht="30">
       <c r="A9" s="6">
         <v>8</v>
       </c>
       <c r="B9" s="6" t="s">
+        <v>15</v>
+      </c>
+      <c r="C9" s="6" t="s">
         <v>18</v>
       </c>
-      <c r="C9" s="6" t="s">
-        <v>23</v>
-      </c>
       <c r="D9" s="7" t="s">
-        <v>24</v>
+        <v>19</v>
       </c>
       <c r="E9" s="8" t="s">
         <v>9</v>
@@ -1198,13 +1157,13 @@
         <v>9</v>
       </c>
       <c r="B10" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>25</v>
+        <v>20</v>
       </c>
       <c r="D10" s="7" t="s">
-        <v>26</v>
+        <v>21</v>
       </c>
       <c r="E10" s="8" t="s">
         <v>9</v>
@@ -1216,13 +1175,13 @@
         <v>10</v>
       </c>
       <c r="B11" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>27</v>
+        <v>22</v>
       </c>
       <c r="D11" s="7" t="s">
-        <v>28</v>
+        <v>23</v>
       </c>
       <c r="E11" s="8" t="s">
         <v>9</v>
@@ -1234,13 +1193,13 @@
         <v>11</v>
       </c>
       <c r="B12" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>29</v>
+        <v>24</v>
       </c>
       <c r="D12" s="7" t="s">
-        <v>30</v>
+        <v>25</v>
       </c>
       <c r="E12" s="8" t="s">
         <v>9</v>
@@ -1252,31 +1211,31 @@
         <v>12</v>
       </c>
       <c r="B13" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>31</v>
+        <v>26</v>
       </c>
       <c r="D13" s="7" t="s">
-        <v>32</v>
+        <v>27</v>
       </c>
       <c r="E13" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F13" s="7"/>
     </row>
-    <row r="14" spans="1:6" ht="30">
+    <row r="14" spans="1:6">
       <c r="A14" s="6">
         <v>13</v>
       </c>
       <c r="B14" s="6" t="s">
-        <v>18</v>
+        <v>15</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>33</v>
+        <v>28</v>
       </c>
       <c r="D14" s="7" t="s">
-        <v>34</v>
+        <v>29</v>
       </c>
       <c r="E14" s="8" t="s">
         <v>9</v>
@@ -1288,13 +1247,13 @@
         <v>14</v>
       </c>
       <c r="B15" s="6" t="s">
-        <v>35</v>
+        <v>15</v>
       </c>
       <c r="C15" s="6" t="s">
-        <v>36</v>
+        <v>30</v>
       </c>
       <c r="D15" s="7" t="s">
-        <v>37</v>
+        <v>31</v>
       </c>
       <c r="E15" s="8" t="s">
         <v>9</v>
@@ -1306,13 +1265,13 @@
         <v>15</v>
       </c>
       <c r="B16" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C16" s="6" t="s">
-        <v>38</v>
+        <v>33</v>
       </c>
       <c r="D16" s="7" t="s">
-        <v>39</v>
+        <v>34</v>
       </c>
       <c r="E16" s="8" t="s">
         <v>9</v>
@@ -1324,13 +1283,13 @@
         <v>16</v>
       </c>
       <c r="B17" s="6" t="s">
+        <v>32</v>
+      </c>
+      <c r="C17" s="6" t="s">
         <v>35</v>
       </c>
-      <c r="C17" s="6" t="s">
-        <v>40</v>
-      </c>
       <c r="D17" s="7" t="s">
-        <v>41</v>
+        <v>36</v>
       </c>
       <c r="E17" s="8" t="s">
         <v>9</v>
@@ -1342,13 +1301,13 @@
         <v>17</v>
       </c>
       <c r="B18" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C18" s="6" t="s">
-        <v>42</v>
+        <v>37</v>
       </c>
       <c r="D18" s="7" t="s">
-        <v>43</v>
+        <v>38</v>
       </c>
       <c r="E18" s="8" t="s">
         <v>9</v>
@@ -1360,49 +1319,49 @@
         <v>18</v>
       </c>
       <c r="B19" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C19" s="6" t="s">
-        <v>44</v>
+        <v>39</v>
       </c>
       <c r="D19" s="7" t="s">
-        <v>45</v>
+        <v>40</v>
       </c>
       <c r="E19" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F19" s="7"/>
     </row>
-    <row r="20" spans="1:6">
+    <row r="20" spans="1:6" ht="30">
       <c r="A20" s="6">
         <v>19</v>
       </c>
       <c r="B20" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C20" s="6" t="s">
-        <v>46</v>
+        <v>41</v>
       </c>
       <c r="D20" s="7" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="E20" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F20" s="7"/>
     </row>
-    <row r="21" spans="1:6" ht="30">
+    <row r="21" spans="1:6">
       <c r="A21" s="6">
         <v>20</v>
       </c>
       <c r="B21" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C21" s="6" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="D21" s="7" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="E21" s="8" t="s">
         <v>9</v>
@@ -1414,31 +1373,31 @@
         <v>21</v>
       </c>
       <c r="B22" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C22" s="6" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="D22" s="7" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="E22" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F22" s="7"/>
     </row>
-    <row r="23" spans="1:6">
+    <row r="23" spans="1:6" ht="30">
       <c r="A23" s="6">
         <v>22</v>
       </c>
       <c r="B23" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C23" s="6" t="s">
-        <v>52</v>
+        <v>47</v>
       </c>
       <c r="D23" s="7" t="s">
-        <v>53</v>
+        <v>48</v>
       </c>
       <c r="E23" s="8" t="s">
         <v>9</v>
@@ -1450,67 +1409,67 @@
         <v>23</v>
       </c>
       <c r="B24" s="6" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C24" s="6" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="D24" s="7" t="s">
-        <v>55</v>
+        <v>50</v>
       </c>
       <c r="E24" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F24" s="7"/>
     </row>
-    <row r="25" spans="1:6" ht="30">
+    <row r="25" spans="1:6">
       <c r="A25" s="6">
         <v>24</v>
       </c>
       <c r="B25" s="6" t="s">
-        <v>56</v>
+        <v>32</v>
       </c>
       <c r="C25" s="6" t="s">
-        <v>57</v>
+        <v>51</v>
       </c>
       <c r="D25" s="7" t="s">
-        <v>58</v>
+        <v>52</v>
       </c>
       <c r="E25" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F25" s="7"/>
     </row>
-    <row r="26" spans="1:6" ht="30">
+    <row r="26" spans="1:6" ht="60">
       <c r="A26" s="6">
         <v>25</v>
       </c>
       <c r="B26" s="6" t="s">
-        <v>56</v>
+        <v>169</v>
       </c>
       <c r="C26" s="6" t="s">
-        <v>59</v>
+        <v>170</v>
       </c>
       <c r="D26" s="7" t="s">
-        <v>60</v>
+        <v>171</v>
       </c>
       <c r="E26" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F26" s="7"/>
     </row>
-    <row r="27" spans="1:6" ht="30">
+    <row r="27" spans="1:6" ht="45">
       <c r="A27" s="6">
         <v>26</v>
       </c>
       <c r="B27" s="6" t="s">
-        <v>56</v>
+        <v>169</v>
       </c>
       <c r="C27" s="6" t="s">
-        <v>61</v>
+        <v>172</v>
       </c>
       <c r="D27" s="7" t="s">
-        <v>62</v>
+        <v>173</v>
       </c>
       <c r="E27" s="8" t="s">
         <v>9</v>
@@ -1522,13 +1481,13 @@
         <v>27</v>
       </c>
       <c r="B28" s="6" t="s">
-        <v>56</v>
+        <v>169</v>
       </c>
       <c r="C28" s="6" t="s">
-        <v>63</v>
+        <v>174</v>
       </c>
       <c r="D28" s="7" t="s">
-        <v>64</v>
+        <v>175</v>
       </c>
       <c r="E28" s="8" t="s">
         <v>9</v>
@@ -1540,13 +1499,13 @@
         <v>28</v>
       </c>
       <c r="B29" s="6" t="s">
-        <v>56</v>
+        <v>169</v>
       </c>
       <c r="C29" s="6" t="s">
-        <v>65</v>
+        <v>176</v>
       </c>
       <c r="D29" s="7" t="s">
-        <v>66</v>
+        <v>177</v>
       </c>
       <c r="E29" s="8" t="s">
         <v>9</v>
@@ -1558,49 +1517,49 @@
         <v>29</v>
       </c>
       <c r="B30" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C30" s="6" t="s">
-        <v>67</v>
+        <v>54</v>
       </c>
       <c r="D30" s="7" t="s">
-        <v>68</v>
+        <v>55</v>
       </c>
       <c r="E30" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F30" s="7"/>
     </row>
-    <row r="31" spans="1:6">
+    <row r="31" spans="1:6" ht="30">
       <c r="A31" s="6">
         <v>30</v>
       </c>
       <c r="B31" s="6" t="s">
+        <v>53</v>
+      </c>
+      <c r="C31" s="6" t="s">
         <v>56</v>
       </c>
-      <c r="C31" s="6" t="s">
-        <v>69</v>
-      </c>
       <c r="D31" s="7" t="s">
-        <v>70</v>
+        <v>57</v>
       </c>
       <c r="E31" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F31" s="7"/>
     </row>
-    <row r="32" spans="1:6">
+    <row r="32" spans="1:6" ht="30">
       <c r="A32" s="6">
         <v>31</v>
       </c>
       <c r="B32" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C32" s="6" t="s">
-        <v>71</v>
+        <v>58</v>
       </c>
       <c r="D32" s="7" t="s">
-        <v>72</v>
+        <v>59</v>
       </c>
       <c r="E32" s="8" t="s">
         <v>9</v>
@@ -1612,13 +1571,13 @@
         <v>32</v>
       </c>
       <c r="B33" s="6" t="s">
-        <v>56</v>
+        <v>53</v>
       </c>
       <c r="C33" s="6" t="s">
-        <v>73</v>
+        <v>60</v>
       </c>
       <c r="D33" s="7" t="s">
-        <v>74</v>
+        <v>61</v>
       </c>
       <c r="E33" s="8" t="s">
         <v>9</v>
@@ -1630,13 +1589,13 @@
         <v>33</v>
       </c>
       <c r="B34" s="6" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C34" s="6" t="s">
-        <v>76</v>
+        <v>62</v>
       </c>
       <c r="D34" s="7" t="s">
-        <v>77</v>
+        <v>63</v>
       </c>
       <c r="E34" s="8" t="s">
         <v>9</v>
@@ -1648,49 +1607,49 @@
         <v>34</v>
       </c>
       <c r="B35" s="6" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C35" s="6" t="s">
-        <v>78</v>
+        <v>64</v>
       </c>
       <c r="D35" s="7" t="s">
-        <v>79</v>
+        <v>65</v>
       </c>
       <c r="E35" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F35" s="7"/>
     </row>
-    <row r="36" spans="1:6" ht="30">
+    <row r="36" spans="1:6">
       <c r="A36" s="6">
         <v>35</v>
       </c>
       <c r="B36" s="6" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C36" s="6" t="s">
-        <v>80</v>
+        <v>66</v>
       </c>
       <c r="D36" s="7" t="s">
-        <v>81</v>
+        <v>67</v>
       </c>
       <c r="E36" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F36" s="7"/>
     </row>
-    <row r="37" spans="1:6" ht="30">
+    <row r="37" spans="1:6">
       <c r="A37" s="6">
         <v>36</v>
       </c>
       <c r="B37" s="6" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C37" s="6" t="s">
-        <v>82</v>
+        <v>68</v>
       </c>
       <c r="D37" s="7" t="s">
-        <v>83</v>
+        <v>69</v>
       </c>
       <c r="E37" s="8" t="s">
         <v>9</v>
@@ -1702,13 +1661,13 @@
         <v>37</v>
       </c>
       <c r="B38" s="6" t="s">
-        <v>75</v>
+        <v>53</v>
       </c>
       <c r="C38" s="6" t="s">
-        <v>84</v>
+        <v>70</v>
       </c>
       <c r="D38" s="7" t="s">
-        <v>85</v>
+        <v>71</v>
       </c>
       <c r="E38" s="8" t="s">
         <v>9</v>
@@ -1720,13 +1679,13 @@
         <v>38</v>
       </c>
       <c r="B39" s="6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="C39" s="6" t="s">
-        <v>86</v>
+        <v>73</v>
       </c>
       <c r="D39" s="7" t="s">
-        <v>87</v>
+        <v>74</v>
       </c>
       <c r="E39" s="8" t="s">
         <v>9</v>
@@ -1738,13 +1697,13 @@
         <v>39</v>
       </c>
       <c r="B40" s="6" t="s">
+        <v>72</v>
+      </c>
+      <c r="C40" s="6" t="s">
         <v>75</v>
       </c>
-      <c r="C40" s="6" t="s">
-        <v>88</v>
-      </c>
       <c r="D40" s="7" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="E40" s="8" t="s">
         <v>9</v>
@@ -1756,13 +1715,13 @@
         <v>40</v>
       </c>
       <c r="B41" s="6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C41" s="6" t="s">
-        <v>91</v>
+        <v>77</v>
       </c>
       <c r="D41" s="7" t="s">
-        <v>92</v>
+        <v>78</v>
       </c>
       <c r="E41" s="8" t="s">
         <v>9</v>
@@ -1774,31 +1733,31 @@
         <v>41</v>
       </c>
       <c r="B42" s="6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C42" s="6" t="s">
-        <v>93</v>
+        <v>79</v>
       </c>
       <c r="D42" s="7" t="s">
-        <v>94</v>
+        <v>80</v>
       </c>
       <c r="E42" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F42" s="7"/>
     </row>
-    <row r="43" spans="1:6">
+    <row r="43" spans="1:6" ht="30">
       <c r="A43" s="6">
         <v>42</v>
       </c>
       <c r="B43" s="6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C43" s="6" t="s">
-        <v>95</v>
+        <v>81</v>
       </c>
       <c r="D43" s="7" t="s">
-        <v>96</v>
+        <v>82</v>
       </c>
       <c r="E43" s="8" t="s">
         <v>9</v>
@@ -1810,49 +1769,49 @@
         <v>43</v>
       </c>
       <c r="B44" s="6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C44" s="6" t="s">
-        <v>97</v>
+        <v>83</v>
       </c>
       <c r="D44" s="7" t="s">
-        <v>98</v>
+        <v>84</v>
       </c>
       <c r="E44" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F44" s="7"/>
     </row>
-    <row r="45" spans="1:6">
+    <row r="45" spans="1:6" ht="30">
       <c r="A45" s="6">
         <v>44</v>
       </c>
       <c r="B45" s="6" t="s">
-        <v>90</v>
+        <v>72</v>
       </c>
       <c r="C45" s="6" t="s">
-        <v>99</v>
+        <v>85</v>
       </c>
       <c r="D45" s="7" t="s">
-        <v>100</v>
+        <v>86</v>
       </c>
       <c r="E45" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F45" s="7"/>
     </row>
-    <row r="46" spans="1:6">
+    <row r="46" spans="1:6" ht="30">
       <c r="A46" s="6">
         <v>45</v>
       </c>
       <c r="B46" s="6" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="C46" s="6" t="s">
-        <v>102</v>
+        <v>88</v>
       </c>
       <c r="D46" s="7" t="s">
-        <v>103</v>
+        <v>89</v>
       </c>
       <c r="E46" s="8" t="s">
         <v>9</v>
@@ -1864,31 +1823,31 @@
         <v>46</v>
       </c>
       <c r="B47" s="6" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="C47" s="6" t="s">
-        <v>104</v>
+        <v>90</v>
       </c>
       <c r="D47" s="7" t="s">
-        <v>105</v>
+        <v>91</v>
       </c>
       <c r="E47" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F47" s="7"/>
     </row>
-    <row r="48" spans="1:6" ht="30">
+    <row r="48" spans="1:6">
       <c r="A48" s="6">
         <v>47</v>
       </c>
       <c r="B48" s="6" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="C48" s="6" t="s">
-        <v>106</v>
+        <v>92</v>
       </c>
       <c r="D48" s="7" t="s">
-        <v>107</v>
+        <v>93</v>
       </c>
       <c r="E48" s="8" t="s">
         <v>9</v>
@@ -1900,13 +1859,13 @@
         <v>48</v>
       </c>
       <c r="B49" s="6" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="C49" s="6" t="s">
-        <v>108</v>
+        <v>94</v>
       </c>
       <c r="D49" s="7" t="s">
-        <v>109</v>
+        <v>95</v>
       </c>
       <c r="E49" s="8" t="s">
         <v>9</v>
@@ -1918,13 +1877,13 @@
         <v>49</v>
       </c>
       <c r="B50" s="6" t="s">
-        <v>101</v>
+        <v>87</v>
       </c>
       <c r="C50" s="6" t="s">
-        <v>110</v>
+        <v>96</v>
       </c>
       <c r="D50" s="7" t="s">
-        <v>111</v>
+        <v>97</v>
       </c>
       <c r="E50" s="8" t="s">
         <v>9</v>
@@ -1936,13 +1895,13 @@
         <v>50</v>
       </c>
       <c r="B51" s="6" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
       <c r="C51" s="6" t="s">
-        <v>112</v>
+        <v>99</v>
       </c>
       <c r="D51" s="7" t="s">
-        <v>113</v>
+        <v>100</v>
       </c>
       <c r="E51" s="8" t="s">
         <v>9</v>
@@ -1954,13 +1913,13 @@
         <v>51</v>
       </c>
       <c r="B52" s="6" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C52" s="6" t="s">
-        <v>115</v>
+        <v>101</v>
       </c>
       <c r="D52" s="7" t="s">
-        <v>116</v>
+        <v>102</v>
       </c>
       <c r="E52" s="8" t="s">
         <v>9</v>
@@ -1972,49 +1931,49 @@
         <v>52</v>
       </c>
       <c r="B53" s="6" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C53" s="6" t="s">
-        <v>117</v>
+        <v>103</v>
       </c>
       <c r="D53" s="7" t="s">
-        <v>118</v>
+        <v>104</v>
       </c>
       <c r="E53" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F53" s="7"/>
     </row>
-    <row r="54" spans="1:6">
+    <row r="54" spans="1:6" ht="30">
       <c r="A54" s="6">
         <v>53</v>
       </c>
       <c r="B54" s="6" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C54" s="6" t="s">
-        <v>119</v>
+        <v>105</v>
       </c>
       <c r="D54" s="7" t="s">
-        <v>120</v>
+        <v>106</v>
       </c>
       <c r="E54" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F54" s="7"/>
     </row>
-    <row r="55" spans="1:6" ht="30">
+    <row r="55" spans="1:6">
       <c r="A55" s="6">
         <v>54</v>
       </c>
       <c r="B55" s="6" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C55" s="6" t="s">
-        <v>121</v>
+        <v>107</v>
       </c>
       <c r="D55" s="7" t="s">
-        <v>122</v>
+        <v>108</v>
       </c>
       <c r="E55" s="8" t="s">
         <v>9</v>
@@ -2026,31 +1985,31 @@
         <v>55</v>
       </c>
       <c r="B56" s="6" t="s">
-        <v>114</v>
+        <v>98</v>
       </c>
       <c r="C56" s="6" t="s">
-        <v>123</v>
+        <v>109</v>
       </c>
       <c r="D56" s="7" t="s">
-        <v>124</v>
+        <v>110</v>
       </c>
       <c r="E56" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F56" s="7"/>
     </row>
-    <row r="57" spans="1:6">
+    <row r="57" spans="1:6" ht="30">
       <c r="A57" s="6">
         <v>56</v>
       </c>
       <c r="B57" s="6" t="s">
-        <v>114</v>
+        <v>111</v>
       </c>
       <c r="C57" s="6" t="s">
-        <v>125</v>
+        <v>112</v>
       </c>
       <c r="D57" s="7" t="s">
-        <v>126</v>
+        <v>113</v>
       </c>
       <c r="E57" s="8" t="s">
         <v>9</v>
@@ -2062,13 +2021,13 @@
         <v>57</v>
       </c>
       <c r="B58" s="6" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C58" s="6" t="s">
-        <v>128</v>
+        <v>114</v>
       </c>
       <c r="D58" s="7" t="s">
-        <v>129</v>
+        <v>115</v>
       </c>
       <c r="E58" s="8" t="s">
         <v>9</v>
@@ -2080,13 +2039,13 @@
         <v>58</v>
       </c>
       <c r="B59" s="6" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C59" s="6" t="s">
-        <v>130</v>
+        <v>116</v>
       </c>
       <c r="D59" s="7" t="s">
-        <v>131</v>
+        <v>117</v>
       </c>
       <c r="E59" s="8" t="s">
         <v>9</v>
@@ -2098,31 +2057,31 @@
         <v>59</v>
       </c>
       <c r="B60" s="6" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C60" s="6" t="s">
-        <v>132</v>
+        <v>118</v>
       </c>
       <c r="D60" s="7" t="s">
-        <v>133</v>
+        <v>119</v>
       </c>
       <c r="E60" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F60" s="7"/>
     </row>
-    <row r="61" spans="1:6" ht="30">
+    <row r="61" spans="1:6">
       <c r="A61" s="6">
         <v>60</v>
       </c>
       <c r="B61" s="6" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C61" s="6" t="s">
-        <v>134</v>
+        <v>120</v>
       </c>
       <c r="D61" s="7" t="s">
-        <v>135</v>
+        <v>121</v>
       </c>
       <c r="E61" s="8" t="s">
         <v>9</v>
@@ -2134,13 +2093,13 @@
         <v>61</v>
       </c>
       <c r="B62" s="6" t="s">
-        <v>127</v>
+        <v>111</v>
       </c>
       <c r="C62" s="6" t="s">
-        <v>136</v>
+        <v>122</v>
       </c>
       <c r="D62" s="7" t="s">
-        <v>137</v>
+        <v>123</v>
       </c>
       <c r="E62" s="8" t="s">
         <v>9</v>
@@ -2152,13 +2111,13 @@
         <v>62</v>
       </c>
       <c r="B63" s="6" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C63" s="6" t="s">
-        <v>139</v>
+        <v>125</v>
       </c>
       <c r="D63" s="7" t="s">
-        <v>140</v>
+        <v>126</v>
       </c>
       <c r="E63" s="8" t="s">
         <v>9</v>
@@ -2170,233 +2129,198 @@
         <v>63</v>
       </c>
       <c r="B64" s="6" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C64" s="6" t="s">
-        <v>141</v>
+        <v>127</v>
       </c>
       <c r="D64" s="7" t="s">
-        <v>142</v>
+        <v>128</v>
       </c>
       <c r="E64" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F64" s="7"/>
     </row>
-    <row r="65" spans="1:7" ht="30">
+    <row r="65" spans="1:6" ht="30">
       <c r="A65" s="6">
         <v>64</v>
       </c>
       <c r="B65" s="6" t="s">
-        <v>138</v>
+        <v>124</v>
       </c>
       <c r="C65" s="6" t="s">
-        <v>143</v>
+        <v>129</v>
       </c>
       <c r="D65" s="7" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="E65" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F65" s="7"/>
     </row>
-    <row r="66" spans="1:7" ht="30">
+    <row r="66" spans="1:6" ht="30">
       <c r="A66" s="6">
         <v>65</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>145</v>
+        <v>124</v>
       </c>
       <c r="C66" s="6" t="s">
-        <v>146</v>
+        <v>131</v>
       </c>
       <c r="D66" s="7" t="s">
-        <v>147</v>
+        <v>132</v>
       </c>
       <c r="E66" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F66" s="7"/>
     </row>
-    <row r="67" spans="1:7">
+    <row r="67" spans="1:6">
       <c r="A67" s="6">
         <v>66</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>145</v>
+        <v>124</v>
       </c>
       <c r="C67" s="6" t="s">
-        <v>148</v>
+        <v>133</v>
       </c>
       <c r="D67" s="7" t="s">
-        <v>149</v>
+        <v>134</v>
       </c>
       <c r="E67" s="8" t="s">
         <v>9</v>
       </c>
       <c r="F67" s="7"/>
     </row>
-    <row r="68" spans="1:7" ht="30">
+    <row r="68" spans="1:6" ht="30">
       <c r="A68" s="6">
         <v>67</v>
       </c>
       <c r="B68" s="6" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="C68" s="6" t="s">
-        <v>150</v>
+        <v>136</v>
       </c>
       <c r="D68" s="7" t="s">
-        <v>151</v>
+        <v>137</v>
       </c>
       <c r="E68" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F68" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="G68" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="69" spans="1:7" ht="30">
+      <c r="F68" s="7"/>
+    </row>
+    <row r="69" spans="1:6">
       <c r="A69" s="6">
         <v>68</v>
       </c>
       <c r="B69" s="6" t="s">
-        <v>114</v>
+        <v>135</v>
       </c>
       <c r="C69" s="6" t="s">
-        <v>152</v>
+        <v>138</v>
       </c>
       <c r="D69" s="7" t="s">
-        <v>153</v>
+        <v>139</v>
       </c>
       <c r="E69" s="8" t="s">
         <v>9</v>
       </c>
-      <c r="F69" s="7" t="s">
-        <v>168</v>
-      </c>
-      <c r="G69" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="70" spans="1:7" ht="165">
-      <c r="A70" s="12">
+      <c r="F69" s="7"/>
+    </row>
+    <row r="70" spans="1:6" ht="30">
+      <c r="A70" s="6">
         <v>69</v>
       </c>
-      <c r="B70" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C70" s="12" t="s">
-        <v>172</v>
-      </c>
-      <c r="D70" s="13" t="s">
-        <v>173</v>
-      </c>
-      <c r="E70" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="F70" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G70" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="71" spans="1:7" ht="165">
-      <c r="A71" s="12">
+      <c r="B70" s="6" t="s">
+        <v>135</v>
+      </c>
+      <c r="C70" s="6" t="s">
+        <v>140</v>
+      </c>
+      <c r="D70" s="7" t="s">
+        <v>141</v>
+      </c>
+      <c r="E70" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F70" s="7"/>
+    </row>
+    <row r="71" spans="1:6" ht="30">
+      <c r="A71" s="6">
         <v>70</v>
       </c>
-      <c r="B71" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C71" s="12" t="s">
-        <v>177</v>
-      </c>
-      <c r="D71" s="13" t="s">
-        <v>178</v>
-      </c>
-      <c r="E71" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="F71" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G71" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="72" spans="1:7" ht="165">
-      <c r="A72" s="12">
+      <c r="B71" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C71" s="6" t="s">
+        <v>143</v>
+      </c>
+      <c r="D71" s="7" t="s">
+        <v>144</v>
+      </c>
+      <c r="E71" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F71" s="7"/>
+    </row>
+    <row r="72" spans="1:6">
+      <c r="A72" s="6">
         <v>71</v>
       </c>
-      <c r="B72" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C72" s="12" t="s">
-        <v>179</v>
-      </c>
-      <c r="D72" s="13" t="s">
-        <v>180</v>
-      </c>
-      <c r="E72" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="F72" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G72" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="73" spans="1:7" ht="165">
-      <c r="A73" s="12">
+      <c r="B72" s="6" t="s">
+        <v>142</v>
+      </c>
+      <c r="C72" s="6" t="s">
+        <v>145</v>
+      </c>
+      <c r="D72" s="7" t="s">
+        <v>146</v>
+      </c>
+      <c r="E72" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F72" s="7"/>
+    </row>
+    <row r="73" spans="1:6" ht="30">
+      <c r="A73" s="6">
         <v>72</v>
       </c>
-      <c r="B73" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C73" s="12" t="s">
-        <v>181</v>
-      </c>
-      <c r="D73" s="13" t="s">
-        <v>182</v>
-      </c>
-      <c r="E73" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="F73" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G73" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="74" spans="1:7" ht="165">
-      <c r="A74" s="12">
+      <c r="B73" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C73" s="6" t="s">
+        <v>147</v>
+      </c>
+      <c r="D73" s="7" t="s">
+        <v>148</v>
+      </c>
+      <c r="E73" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F73" s="7"/>
+    </row>
+    <row r="74" spans="1:6" ht="30">
+      <c r="A74" s="6">
         <v>73</v>
       </c>
-      <c r="B74" s="12" t="s">
-        <v>171</v>
-      </c>
-      <c r="C74" s="12" t="s">
-        <v>183</v>
-      </c>
-      <c r="D74" s="13" t="s">
-        <v>184</v>
-      </c>
-      <c r="E74" s="14" t="s">
-        <v>174</v>
-      </c>
-      <c r="F74" s="13" t="s">
-        <v>175</v>
-      </c>
-      <c r="G74" s="3" t="s">
-        <v>176</v>
-      </c>
+      <c r="B74" s="6" t="s">
+        <v>111</v>
+      </c>
+      <c r="C74" s="6" t="s">
+        <v>149</v>
+      </c>
+      <c r="D74" s="7" t="s">
+        <v>150</v>
+      </c>
+      <c r="E74" s="8" t="s">
+        <v>9</v>
+      </c>
+      <c r="F74" s="7"/>
     </row>
   </sheetData>
   <autoFilter ref="A1:F1"/>
@@ -2416,12 +2340,12 @@
   <sheetData>
     <row r="1" spans="1:2" ht="21">
       <c r="A1" s="9" t="s">
-        <v>154</v>
+        <v>151</v>
       </c>
     </row>
     <row r="2" spans="1:2">
       <c r="A2" s="10" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
     </row>
     <row r="4" spans="1:2">
@@ -2429,21 +2353,21 @@
         <v>4</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>156</v>
+        <v>153</v>
       </c>
     </row>
     <row r="5" spans="1:2">
       <c r="A5" s="11" t="s">
-        <v>157</v>
+        <v>154</v>
       </c>
       <c r="B5" s="11">
         <f>COUNTIF('Feature Tracker'!E:E,"Completed")</f>
-        <v>68</v>
+        <v>73</v>
       </c>
     </row>
     <row r="6" spans="1:2">
       <c r="A6" s="11" t="s">
-        <v>158</v>
+        <v>155</v>
       </c>
       <c r="B6" s="11">
         <f>COUNTIF('Feature Tracker'!E:E,"Planned")</f>
@@ -2452,51 +2376,51 @@
     </row>
     <row r="7" spans="1:2">
       <c r="A7" s="11" t="s">
-        <v>159</v>
+        <v>156</v>
       </c>
       <c r="B7" s="11">
         <f>COUNTIF('Feature Tracker'!E:E,"Proposed")</f>
-        <v>5</v>
+        <v>0</v>
       </c>
     </row>
     <row r="9" spans="1:2">
       <c r="A9" s="1" t="s">
-        <v>160</v>
+        <v>157</v>
       </c>
     </row>
     <row r="10" spans="1:2">
       <c r="A10" t="s">
-        <v>161</v>
+        <v>158</v>
       </c>
     </row>
     <row r="11" spans="1:2">
       <c r="A11" t="s">
-        <v>162</v>
+        <v>159</v>
       </c>
     </row>
     <row r="12" spans="1:2">
       <c r="A12" t="s">
-        <v>163</v>
+        <v>160</v>
       </c>
     </row>
     <row r="13" spans="1:2">
       <c r="A13" t="s">
-        <v>164</v>
+        <v>161</v>
       </c>
     </row>
     <row r="14" spans="1:2">
       <c r="A14" t="s">
-        <v>165</v>
+        <v>162</v>
       </c>
     </row>
     <row r="15" spans="1:2">
       <c r="A15" t="s">
-        <v>166</v>
+        <v>163</v>
       </c>
     </row>
     <row r="16" spans="1:2">
       <c r="A16" t="s">
-        <v>167</v>
+        <v>164</v>
       </c>
     </row>
   </sheetData>

</xml_diff>